<commit_message>
Scenarios workbook: update Instructions title, approval record and app-figure note
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/chat_british_scenarios.xlsx
+++ b/data/chat_british_scenarios.xlsx
@@ -576,7 +576,7 @@
     <row r="1" ht="16.15" customHeight="1" s="15">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Chat British: Practice scenarios (114 + the 6 already in the app = 120)</t>
+          <t>Chat British: Practice scenarios (120)</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>All rows are Approved because the founder accepted the whole set. The Review state column records what that means: 18 rows (batch 1) were read and approved individually; the other 96 were accepted in bulk and still need an item-by-item read. Please change Review state to "Reviewed and approved by founder" as you go. Do not remove the column.</t>
+          <t>All rows are Approved because the founder accepted the whole set. The Review state column records what that means: 24 rows (the original 6 and batch 1) were read and approved individually; the other 96 were accepted in bulk and still need an item-by-item read. Please change Review state to "Reviewed and approved by founder" as you go. Do not remove the column.</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>Input: the six scenarios already in the app, which Cursor migrates into this workbook.</t>
+          <t>All scenarios now live in this workbook.</t>
         </is>
       </c>
     </row>

</xml_diff>